<commit_message>
Nhập theo trường: nhiều cuộc thi trong một dòng, chia lệ phí theo giá
- Tách "FIMO & FIEO & SIAIO", "A, B và C", "A - B", "A | B"... thành
  từng cuộc thi; trước đây "A - B" chỉ khớp cuộc thi đầu.
- Lệ phí chung của dòng được chia theo giá từng cuộc thi học từ các dòng
  đăng ký một cuộc thi trong cùng file; không có thì chia đều nếu chia hết,
  còn lại chỉ bỏ qua dòng đó.
- File mẫu bỏ danh sách chọn cố định ở cột Cuộc thi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/Mau_dang_ky_theo_truong.xlsx
+++ b/public/templates/Mau_dang_ky_theo_truong.xlsx
@@ -3449,11 +3449,6 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C5:I5"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="F13:F212" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"FIMO,FIEO,FIMO &amp; FIEO"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3554,7 +3549,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ghi FIMO, FIEO hoặc FIMO &amp; FIEO nếu thí sinh đăng ký cả hai cuộc thi.</t>
+          <t>Ghi một hoặc nhiều mã, nối bằng &amp; hoặc dấu phẩy. VD: FIMO &amp; FIEO &amp; SIAIO.</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3561,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ghi tổng lệ phí của dòng (VD 500.000 cho FIMO &amp; FIEO); hệ thống tự chia đều cho từng cuộc thi.</t>
+          <t>Ghi tổng lệ phí của dòng. Hệ thống chia theo giá từng cuộc thi (lấy từ các dòng chỉ đăng ký một cuộc thi), không có thì chia đều.</t>
         </is>
       </c>
     </row>

</xml_diff>